<commit_message>
Améliore le SEO et la navigation
</commit_message>
<xml_diff>
--- a/downloads/CyberReperes_Catalogue_Methodes.xlsx
+++ b/downloads/CyberReperes_Catalogue_Methodes.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Menaces" sheetId="1" state="visible" r:id="rId2"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="197">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -113,175 +113,178 @@
     <t xml:space="preserve">THR-003</t>
   </si>
   <si>
+    <t xml:space="preserve">CERT-FR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">État de la menace au travers de bulletins du CERT-FR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Priorisation et réduction de l'exposition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IT / OT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alertes en cours, Avis de Sécurité, IOC, bulletin d’actualité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Catalogue vivant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.cert.ssi.gouv.fr/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modèle / outil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Domaines / structure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Niveau / échelle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outil disponible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAT-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U.S. Department of Energy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2M2 – Cybersecurity Capability Maturity Model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Évaluation et amélioration de la capacité cybersécurité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 domaines, objectifs et pratiques</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MIL 1 Initiated / MIL 2 Performed / MIL 3 Managed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Self-Evaluation Tool HTML et PDF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">v2.1 – juin 2022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.energy.gov/ceser/cybersecurity-capability-maturity-model-c2m2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Très pertinent pour OT énergie mais utilisable plus largement.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAT-002</t>
+  </si>
+  <si>
     <t xml:space="preserve">CISA</t>
   </si>
   <si>
+    <t xml:space="preserve">Cybersecurity Performance Goals (CPGs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Socle de pratiques prioritaires de cybersécurité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IT / OT / CNI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Objectifs et pratiques prioritaires</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pas un modèle de maturité classique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ressource web</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Évolutif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.cisa.gov/cybersecurity-performance-goals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">À ne pas présenter comme un modèle de maturité au même titre que C2M2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Données / sortie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VUL-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FIRST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CVSS v4.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Évaluation de la sévérité technique d'une vulnérabilité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scoring et priorisation des vulnérabilités</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Score CVSS et vecteur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">v4.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.first.org/cvss/v4.0/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ne constitue pas à lui seul une analyse de risque métier.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VUL-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EPSS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimation de la probabilité qu'une vulnérabilité soit exploitée</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Priorisation de la remédiation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Score de probabilité d'exploitation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Service vivant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.first.org/epss/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">À croiser avec CVSS, exposition, criticité et contexte.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VUL-003</t>
+  </si>
+  <si>
     <t xml:space="preserve">Known Exploited Vulnerabilities (KEV) Catalog</t>
   </si>
   <si>
-    <t xml:space="preserve">Catalogue de vulnérabilités connues comme exploitées</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IT / OT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Priorisation de la remédiation et suivi des vulnérabilités exploitées</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Catalogue vivant</t>
+    <t xml:space="preserve">Identification des CVE exploitées dans la nature</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Liste de CVE + échéances / métadonnées</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.cisa.gov/known-exploited-vulnerabilities-catalog</t>
   </si>
   <si>
-    <t xml:space="preserve">À classer aussi dans Vulnérabilités.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modèle / outil</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Domaines / structure</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Niveau / échelle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Outil disponible</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MAT-001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U.S. Department of Energy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C2M2 – Cybersecurity Capability Maturity Model</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Évaluation et amélioration de la capacité cybersécurité</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10 domaines, objectifs et pratiques</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MIL 1 Initiated / MIL 2 Performed / MIL 3 Managed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Self-Evaluation Tool HTML et PDF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">v2.1 – juin 2022</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.energy.gov/ceser/cybersecurity-capability-maturity-model-c2m2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Très pertinent pour OT énergie mais utilisable plus largement.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MAT-002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cybersecurity Performance Goals (CPGs)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Socle de pratiques prioritaires de cybersécurité</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IT / OT / CNI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Objectifs et pratiques prioritaires</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pas un modèle de maturité classique</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ressource web</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Évolutif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.cisa.gov/cybersecurity-performance-goals</t>
-  </si>
-  <si>
-    <t xml:space="preserve">À ne pas présenter comme un modèle de maturité au même titre que C2M2.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Données / sortie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VUL-001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FIRST</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CVSS v4.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Évaluation de la sévérité technique d'une vulnérabilité</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Scoring et priorisation des vulnérabilités</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Score CVSS et vecteur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">v4.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.first.org/cvss/v4.0/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ne constitue pas à lui seul une analyse de risque métier.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VUL-002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EPSS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estimation de la probabilité qu'une vulnérabilité soit exploitée</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Priorisation de la remédiation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Score de probabilité d'exploitation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Service vivant</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.first.org/epss/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">À croiser avec CVSS, exposition, criticité et contexte.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VUL-003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Identification des CVE exploitées dans la nature</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Priorisation et réduction de l'exposition</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Liste de CVE + échéances / métadonnées</t>
-  </si>
-  <si>
     <t xml:space="preserve">À croiser avec le contexte réel de l'actif.</t>
   </si>
   <si>
     <t xml:space="preserve">VUL-004</t>
   </si>
   <si>
-    <t xml:space="preserve">CVE / CVE Program</t>
+    <t xml:space="preserve">Organisme : CVE Program</t>
   </si>
   <si>
     <t xml:space="preserve">Identifiants normalisés de vulnérabilités</t>
@@ -305,18 +308,9 @@
     <t xml:space="preserve">VUL-005</t>
   </si>
   <si>
-    <t xml:space="preserve">CERT-FR</t>
-  </si>
-  <si>
     <t xml:space="preserve">Etat de la menace au travers de bulletins du CERT-FR</t>
   </si>
   <si>
-    <t xml:space="preserve">Alertes en cours, Avis de Sécurité, IOC, bulletin d’actualité</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.cert.ssi.gouv.fr/</t>
-  </si>
-  <si>
     <t xml:space="preserve">Couverture</t>
   </si>
   <si>
@@ -470,12 +464,18 @@
     <t xml:space="preserve">Outil web</t>
   </si>
   <si>
-    <t xml:space="preserve">https://mitre-attack.github.io/attack-navigator/</t>
+    <t xml:space="preserve">https://attack.mitre.org/resources/attack-data-and-tools/</t>
   </si>
   <si>
     <t xml:space="preserve">Complément à ATT&amp;CK, pas un référentiel indépendant.</t>
   </si>
   <si>
+    <t xml:space="preserve">EVA-004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IT / OT / Infra critique</t>
+  </si>
+  <si>
     <t xml:space="preserve">ARC-001</t>
   </si>
   <si>
@@ -491,25 +491,13 @@
     <t xml:space="preserve">Framework, Architecture, segmentation, et maturité</t>
   </si>
   <si>
-    <t xml:space="preserve">Outil</t>
+    <t xml:space="preserve">Référentiel d'architecture</t>
   </si>
   <si>
     <t xml:space="preserve">https://opensecurityarchitecture.org/</t>
   </si>
   <si>
     <t xml:space="preserve">À articuler avec les réalités OT et la segmentation.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARC-002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ATT&amp;CK for ICS Navigator / Matrix</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cartographie des techniques adverses ICS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Threat modeling et couverture de détection</t>
   </si>
   <si>
     <t xml:space="preserve">Famille</t>
@@ -648,7 +636,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -678,12 +666,6 @@
       <name val="Cambria"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
@@ -748,28 +730,32 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -909,135 +895,139 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="48"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="2"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="I2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+    <row r="4" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="G4" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="I4" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="I4" s="2" t="s">
-        <v>32</v>
-      </c>
+      <c r="J4" s="1"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I4"/>
+  <hyperlinks>
+    <hyperlink ref="I4" r:id="rId1" display="https://www.cert.ssi.gouv.fr/"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1045,7 +1035,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -1057,120 +1047,121 @@
   <dimension ref="A1:K3"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="72.23"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="K2" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="K2" s="2" t="s">
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J3" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K3" s="3" t="s">
         <v>56</v>
       </c>
     </row>
@@ -1195,205 +1186,205 @@
   <dimension ref="A1:J6"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="3" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J3" s="3" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="F4" s="2" t="s">
+      <c r="C6" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="H4" s="2" t="s">
+      <c r="G6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H6" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I6" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B6" s="0" t="s">
-        <v>89</v>
-      </c>
-      <c r="C6" s="0" t="s">
-        <v>89</v>
-      </c>
-      <c r="D6" s="0" t="s">
-        <v>90</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="G6" s="0" t="s">
-        <v>91</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="I6" s="0" t="s">
-        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -1420,144 +1411,144 @@
   <dimension ref="A1:J4"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="55"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="H2" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="I2" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="J2" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="I2" s="2" t="s">
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="E3" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="G3" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="F3" s="2" t="s">
+      <c r="H3" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="I3" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="J3" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="H3" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="I3" s="2" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="E4" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="F4" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="G4" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="H4" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="I4" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="J4" s="3" t="s">
         <v>119</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -1578,148 +1569,186 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="55"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="H2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="J2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="B3" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="H4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="J2" s="2"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="F4" s="2" t="s">
+      <c r="I4" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="J4" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="H4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I4" s="2" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="25.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="B5" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>145</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:J4"/>
+  <hyperlinks>
+    <hyperlink ref="I4" r:id="rId1" display="https://attack.mitre.org/resources/attack-data-and-tools/"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1727,7 +1756,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -1739,111 +1768,93 @@
   <dimension ref="A1:J3"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="55"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="H1" s="1" t="s">
+      <c r="G1" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="F2" s="2" t="s">
+      <c r="E2" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="3" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J3" s="2"/>
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J3"/>
@@ -1869,107 +1880,107 @@
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="70"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C2" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D2" s="3" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D6" s="3" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D7" s="3" t="s">
         <v>181</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>185</v>
       </c>
     </row>
   </sheetData>
@@ -1993,104 +2004,104 @@
   <dimension ref="A1:B19"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="105"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="105"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
-        <v>162</v>
-      </c>
-      <c r="B11" s="0" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
-        <v>166</v>
-      </c>
-      <c r="B12" s="0" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
-        <v>170</v>
-      </c>
-      <c r="B13" s="0" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
-        <v>174</v>
-      </c>
-      <c r="B14" s="0" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="s">
         <v>196</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
-        <v>178</v>
-      </c>
-      <c r="B15" s="0" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
-        <v>182</v>
-      </c>
-      <c r="B16" s="0" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
-        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>